<commit_message>
AI Mini Drama iOS: P9 full run, eBug batch, v6 drafts, WDA and log rules
- P9 full run results, ledger, report and run plan; WDA debug notes
- 2026-10-27 P9 eBug batch: drafts, review page, log excerpts, filed codes
- v6 history, drafts with annotation trace and spec agent gaps, comparison
- scripts: annotations.ts, spec-agent-gaps.ts; device.ts restart/blocker,
  check.ts, plan page and usage log updates
- Skills and AGENTS.md: log excerpt attachments on failure entries,
  keeping WDA alive

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/library/ai-mini-drama/ios/cases.xlsx
+++ b/library/ai-mini-drama/ios/cases.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2924" uniqueCount="1761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="1791">
   <si>
     <t>ID</t>
   </si>
@@ -5243,6 +5243,96 @@
     <t>PM error board, 10/13 update (5xxx cards drop the ⓘ). §13.7 card text: 「Couldn't create video. Our service is busy right now. Your credits have been refunded. Try again later.」</t>
   </si>
   <si>
+    <t>TC-364</t>
+  </si>
+  <si>
+    <t>Drama created with 「No captions」; Log stage timings ON</t>
+  </si>
+  <si>
+    <t>Generate the full video; when it finishes, pull the logs and read this video's tool calls</t>
+  </si>
+  <si>
+    <t>The video has no captions, and the log shows no speech-to-text (STT) call for it</t>
+  </si>
+  <si>
+    <t>PM §13.13 (10/6): 「user 選 No captions 時不跑STT」. TC-097 checks the video; this row checks STT did not run. If no log line marks STT on a captioned video either, record Blocked (observability) and ask RD which line does. Spec agent 1012-PM-CAPTIONS-NO-STT (REQ-031)</t>
+  </si>
+  <si>
+    <t>TC-365</t>
+  </si>
+  <si>
+    <t>Captions failed on some segments only (「Captions couldn't be added. Try again」); Log stage timings ON</t>
+  </si>
+  <si>
+    <t>Tap Try again; when the captions appear, pull the logs and compare the STT calls before and after the retry</t>
+  </si>
+  <si>
+    <t>The retry sends only the segments that failed to STT again; the captions appear all at once when every segment has succeeded</t>
+  </si>
+  <si>
+    <t>PM §13.13 (10/6): 「只重跑失敗的段落，全部成功才把字幕一次放上去」. No fault switch makes STT fail (TC-298) → Blocked (observability) until RD gives a fixture. Spec agent 1012-PM-CAPTION-RETRY-SEGMENTS (REQ-031)</t>
+  </si>
+  <si>
+    <t>TC-366</t>
+  </si>
+  <si>
+    <t>Make your character open; a reference photo with an easily recognized object near one edge</t>
+  </si>
+  <si>
+    <t>Add the photo, crop the edge object away in Crop and tap ✓, then Generate; afterwards pull the logs and open the stored reference image (ai-mini-drama-reference-photos)</t>
+  </si>
+  <si>
+    <t>The reference image used for the character shows only the cropped area: the cropped-away object is not in it</t>
+  </si>
+  <si>
+    <t>R-265</t>
+  </si>
+  <si>
+    <t>PM main flow note 「只送 crop 後的圖」 (missed by the first reading; confirmed by a render 2026-10-22). If the pulled logs hold no reference image, record Blocked (observability) and ask RD for the uploaded image. Spec agent 1012-PM-CROP-UPLOAD (REQ-031)</t>
+  </si>
+  <si>
+    <t>TC-367</t>
+  </si>
+  <si>
+    <t>Tier Pro (Pink › IAP › Status › Pro); remaining chats known (finite allowance)</t>
+  </si>
+  <si>
+    <t>Each of the three uses exactly one of the Pro daily chats (allowance 30)</t>
+  </si>
+  <si>
+    <t>MX ① version A. TC-218 runs the same check on any tier; each tier gets its own row (REQ-031). 9999 Developer Server limit → Blocked (chat-count). Spec agent MX-PRO-SEND-DEBIT-001 (REQ-031)</t>
+  </si>
+  <si>
+    <t>TC-368</t>
+  </si>
+  <si>
+    <t>Tier Pro+ (Pink › IAP › Status › Pro+); remaining chats known (finite allowance)</t>
+  </si>
+  <si>
+    <t>Each of the three uses exactly one of the Pro+ daily chats (allowance 100)</t>
+  </si>
+  <si>
+    <t>MX ① version A. TC-218 runs the same check on any tier; each tier gets its own row (REQ-031). 9999 Developer Server limit → Blocked (chat-count). Spec agent MX-PROPLUS-SEND-DEBIT-001 (REQ-031)</t>
+  </si>
+  <si>
+    <t>TC-369</t>
+  </si>
+  <si>
+    <t>RD has changed the Firebase Remote Config daily chat allowance for the tier under test (e.g. Free → 3); app relaunched</t>
+  </si>
+  <si>
+    <t>Send chats until the limit dialog appears, counting each send</t>
+  </si>
+  <si>
+    <t>The limit dialog appears on the send after the new allowance (the 4th for 3), not at the spec default (11th)</t>
+  </si>
+  <si>
+    <t>R-266</t>
+  </si>
+  <si>
+    <t>MX ① version A: allowance is remote-configured (Firebase). The spec does not say when a change takes effect, so relaunch first. Needs RD to change Remote Config → Blocked (remote-config). Spec agent FIXTURE-0924-S002-B016 (REQ-031)</t>
+  </si>
+  <si>
     <t>Feature</t>
   </si>
   <si>
@@ -5264,19 +5354,19 @@
     <t>Version</t>
   </si>
   <si>
-    <t>6</t>
+    <t>7</t>
   </si>
   <si>
     <t>Approved</t>
   </si>
   <si>
-    <t>2026-10-22T03:39:31.188Z</t>
+    <t>2026-10-22T06:29:41.325Z</t>
   </si>
   <si>
     <t>Cases</t>
   </si>
   <si>
-    <t>362</t>
+    <t>368</t>
   </si>
   <si>
     <t>Spec set SHA-256</t>
@@ -5691,7 +5781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H363"/>
+  <dimension ref="A1:H369"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -15138,6 +15228,162 @@
       </c>
       <c r="H363" s="3" t="s">
         <v>1742</v>
+      </c>
+    </row>
+    <row r="364" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A364" s="3" t="s">
+        <v>1743</v>
+      </c>
+      <c r="B364" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C364" s="3" t="s">
+        <v>1744</v>
+      </c>
+      <c r="D364" s="3" t="s">
+        <v>1745</v>
+      </c>
+      <c r="E364" s="3" t="s">
+        <v>1746</v>
+      </c>
+      <c r="F364" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G364" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="H364" s="3" t="s">
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="365" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A365" s="3" t="s">
+        <v>1748</v>
+      </c>
+      <c r="B365" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C365" s="3" t="s">
+        <v>1749</v>
+      </c>
+      <c r="D365" s="3" t="s">
+        <v>1750</v>
+      </c>
+      <c r="E365" s="3" t="s">
+        <v>1751</v>
+      </c>
+      <c r="F365" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G365" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="H365" s="3" t="s">
+        <v>1752</v>
+      </c>
+    </row>
+    <row r="366" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A366" s="3" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B366" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C366" s="3" t="s">
+        <v>1754</v>
+      </c>
+      <c r="D366" s="3" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E366" s="3" t="s">
+        <v>1756</v>
+      </c>
+      <c r="F366" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G366" s="3" t="s">
+        <v>1757</v>
+      </c>
+      <c r="H366" s="3" t="s">
+        <v>1758</v>
+      </c>
+    </row>
+    <row r="367" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A367" s="3" t="s">
+        <v>1759</v>
+      </c>
+      <c r="B367" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="C367" s="3" t="s">
+        <v>1760</v>
+      </c>
+      <c r="D367" s="3" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E367" s="3" t="s">
+        <v>1761</v>
+      </c>
+      <c r="F367" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G367" s="3" t="s">
+        <v>1074</v>
+      </c>
+      <c r="H367" s="3" t="s">
+        <v>1762</v>
+      </c>
+    </row>
+    <row r="368" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A368" s="3" t="s">
+        <v>1763</v>
+      </c>
+      <c r="B368" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="C368" s="3" t="s">
+        <v>1764</v>
+      </c>
+      <c r="D368" s="3" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E368" s="3" t="s">
+        <v>1765</v>
+      </c>
+      <c r="F368" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G368" s="3" t="s">
+        <v>1074</v>
+      </c>
+      <c r="H368" s="3" t="s">
+        <v>1766</v>
+      </c>
+    </row>
+    <row r="369" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A369" s="3" t="s">
+        <v>1767</v>
+      </c>
+      <c r="B369" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="C369" s="3" t="s">
+        <v>1768</v>
+      </c>
+      <c r="D369" s="3" t="s">
+        <v>1769</v>
+      </c>
+      <c r="E369" s="3" t="s">
+        <v>1770</v>
+      </c>
+      <c r="F369" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G369" s="3" t="s">
+        <v>1771</v>
+      </c>
+      <c r="H369" s="3" t="s">
+        <v>1772</v>
       </c>
     </row>
   </sheetData>
@@ -15158,82 +15404,82 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>1743</v>
+        <v>1773</v>
       </c>
       <c r="B1" t="s">
-        <v>1744</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>1745</v>
+        <v>1775</v>
       </c>
       <c r="B2" t="s">
-        <v>1746</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>1747</v>
+        <v>1777</v>
       </c>
       <c r="B3" t="s">
-        <v>1748</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>1749</v>
+        <v>1779</v>
       </c>
       <c r="B4" t="s">
-        <v>1750</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>1751</v>
+        <v>1781</v>
       </c>
       <c r="B5" t="s">
-        <v>1752</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>1753</v>
+        <v>1783</v>
       </c>
       <c r="B6" t="s">
-        <v>1754</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>1755</v>
+        <v>1785</v>
       </c>
       <c r="B7" t="s">
-        <v>1756</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>1757</v>
+        <v>1787</v>
       </c>
       <c r="B8" t="s">
-        <v>1758</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>1757</v>
+        <v>1787</v>
       </c>
       <c r="B9" t="s">
-        <v>1759</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>1757</v>
+        <v>1787</v>
       </c>
       <c r="B10" t="s">
-        <v>1760</v>
+        <v>1790</v>
       </c>
     </row>
   </sheetData>

</xml_diff>